<commit_message>
Final documentation: team names and IDs, light/dark design, illustrations, user guide, task sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EGrnzrfHztmX7RAaosfXYG
</commit_message>
<xml_diff>
--- a/documentation/Nexus_Documentation/Nexus_Feedback_Form.xlsx
+++ b/documentation/Nexus_Documentation/Nexus_Feedback_Form.xlsx
@@ -696,7 +696,7 @@
       <c r="C4" s="42" t="n"/>
       <c r="D4" s="43" t="n"/>
     </row>
-    <row r="5" ht="12.75" customFormat="1" customHeight="1" s="44">
+    <row r="5" ht="80" customFormat="1" customHeight="1" s="44">
       <c r="B5" s="45" t="inlineStr">
         <is>
           <t>Student Details</t>
@@ -709,11 +709,15 @@
       </c>
       <c r="D5" s="47" t="inlineStr">
         <is>
-          <t>[Your name]</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="12.75" customFormat="1" customHeight="1" s="44">
+          <t>Ali Jan
+Humaiz Khan
+Muhammad Ehtisham Shakeel
+Muhammad Waleed
+Ali Turab</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="80" customFormat="1" customHeight="1" s="44">
       <c r="B6" s="48" t="n"/>
       <c r="C6" s="49" t="inlineStr">
         <is>
@@ -722,7 +726,11 @@
       </c>
       <c r="D6" s="50" t="inlineStr">
         <is>
-          <t>[Enrollment no.]</t>
+          <t>Student1661815
+Student1659420
+Student1657963
+Student1659932
+Student1667727</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Documentation: ADSE Semester 3, Aptech Center NN2, system role per team member
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EGrnzrfHztmX7RAaosfXYG
</commit_message>
<xml_diff>
--- a/documentation/Nexus_Documentation/Nexus_Feedback_Form.xlsx
+++ b/documentation/Nexus_Documentation/Nexus_Feedback_Form.xlsx
@@ -743,7 +743,7 @@
       </c>
       <c r="D7" s="52" t="inlineStr">
         <is>
-          <t>[Curriculum]</t>
+          <t>ADSE</t>
         </is>
       </c>
     </row>
@@ -756,7 +756,7 @@
       </c>
       <c r="D8" s="52" t="inlineStr">
         <is>
-          <t>[Semester]</t>
+          <t>Semester 3</t>
         </is>
       </c>
     </row>
@@ -769,7 +769,7 @@
       </c>
       <c r="D9" s="55" t="inlineStr">
         <is>
-          <t>[Centre name]</t>
+          <t>Aptech Center NN2</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       </c>
       <c r="D14" s="63" t="inlineStr">
         <is>
-          <t>[DD/MMM/YYYY]</t>
+          <t>17/Oct/2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Documentation: official centre, course/term, eProject code and project period
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EGrnzrfHztmX7RAaosfXYG
</commit_message>
<xml_diff>
--- a/documentation/Nexus_Documentation/Nexus_Feedback_Form.xlsx
+++ b/documentation/Nexus_Documentation/Nexus_Feedback_Form.xlsx
@@ -743,7 +743,7 @@
       </c>
       <c r="D7" s="52" t="inlineStr">
         <is>
-          <t>ADSE</t>
+          <t>ADSE (ACCP in AI)</t>
         </is>
       </c>
     </row>
@@ -756,7 +756,7 @@
       </c>
       <c r="D8" s="52" t="inlineStr">
         <is>
-          <t>Semester 3</t>
+          <t>Term 3</t>
         </is>
       </c>
     </row>
@@ -769,7 +769,7 @@
       </c>
       <c r="D9" s="55" t="inlineStr">
         <is>
-          <t>Aptech Center NN2</t>
+          <t>ACE-PK-Karachi-20-North Nazimabad-2</t>
         </is>
       </c>
     </row>
@@ -804,7 +804,7 @@
       </c>
       <c r="D12" s="61" t="inlineStr">
         <is>
-          <t>[Duration in days]</t>
+          <t>30 days</t>
         </is>
       </c>
     </row>
@@ -817,7 +817,7 @@
       </c>
       <c r="D13" s="63" t="inlineStr">
         <is>
-          <t>[DD/MMM/YYYY]</t>
+          <t>17/Sep/2026</t>
         </is>
       </c>
     </row>

</xml_diff>